<commit_message>
Sync planning SharePoint : S25
</commit_message>
<xml_diff>
--- a/Plannings 2026 S25 v2.xlsx
+++ b/Plannings 2026 S25 v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cdalpes.sharepoint.com/sites/msteams_bd0f90/Documents partages/02. USP - TOS - General/RH/Plannings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7AA5A74F-8B5F-4333-8824-7AED61442DD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{7AA5A74F-8B5F-4333-8824-7AED61442DD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1F922CC8-FB2A-42B5-8CED-F6F7D790AED3}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="140">
   <si>
     <t>Planning des salariés du 15/06/2026 au 21/06/2026</t>
   </si>
@@ -438,10 +438,10 @@
     <t>17:00/22:20</t>
   </si>
   <si>
-    <t>08:45/17:00</t>
-  </si>
-  <si>
     <t>17:45/23:40</t>
+  </si>
+  <si>
+    <t>08:45/17:45</t>
   </si>
 </sst>
 </file>
@@ -6861,7 +6861,7 @@
         <v>95</v>
       </c>
       <c r="H80" s="56" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.25">
@@ -6893,16 +6893,14 @@
         <v>97</v>
       </c>
       <c r="B83" s="16"/>
-      <c r="C83" s="16"/>
-      <c r="D83" s="16"/>
-      <c r="E83" s="16"/>
-      <c r="F83" s="16"/>
-      <c r="G83" s="16" t="s">
+      <c r="C83" s="59" t="s">
         <v>15</v>
       </c>
-      <c r="H83" s="37" t="s">
-        <v>81</v>
-      </c>
+      <c r="D83" s="60"/>
+      <c r="E83" s="60"/>
+      <c r="F83" s="60"/>
+      <c r="G83" s="60"/>
+      <c r="H83" s="61"/>
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A84" s="65" t="s">
@@ -7017,7 +7015,7 @@
         <v>102</v>
       </c>
       <c r="H91" s="20" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="92" spans="1:8" x14ac:dyDescent="0.25">
@@ -7112,7 +7110,7 @@
       <c r="H98" s="68"/>
     </row>
   </sheetData>
-  <mergeCells count="29">
+  <mergeCells count="30">
     <mergeCell ref="B1:H1"/>
     <mergeCell ref="A5:A6"/>
     <mergeCell ref="A7:A8"/>
@@ -7137,6 +7135,7 @@
     <mergeCell ref="A77:A78"/>
     <mergeCell ref="A79:A82"/>
     <mergeCell ref="A84:A85"/>
+    <mergeCell ref="C83:H83"/>
     <mergeCell ref="B15:H15"/>
     <mergeCell ref="B58:H58"/>
     <mergeCell ref="B56:H56"/>

</xml_diff>